<commit_message>
Read filings missing from companyfacts; ignore non-periodic facts
- sec_crawler: parse the XBRL instance of 10-K/10-Q filings newer than
  companyfacts coverage (adds 2026 Q2 / H1)
- analyze: use only 10-K/10-Q facts (a DEF 14A tagged Medtronic net income
  in millions)
- dashboard: two-line waterfall labels, 10-year cash-flow chart

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/abbott_financials.xlsx
+++ b/data/abbott_financials.xlsx
@@ -3499,7 +3499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV37"/>
+  <dimension ref="A1:AV38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9062,6 +9062,158 @@
       </c>
       <c r="AV37" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026 H1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>half</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>23757000000</v>
+      </c>
+      <c r="G38" t="n">
+        <v>10215000000</v>
+      </c>
+      <c r="H38" t="n">
+        <v>13542000000</v>
+      </c>
+      <c r="I38" t="n">
+        <v>1659000000</v>
+      </c>
+      <c r="J38" t="n">
+        <v>7765000000</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1080000000</v>
+      </c>
+      <c r="L38" t="n">
+        <v>3038000000</v>
+      </c>
+      <c r="M38" t="n">
+        <v>2973000000</v>
+      </c>
+      <c r="N38" t="n">
+        <v>968000000</v>
+      </c>
+      <c r="O38" t="n">
+        <v>2005000000</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0.1049767441860465</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>-0.3540592783505155</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0.5700214673569896</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0.127878099086585</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0.08439617796859873</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0.06983204950119964</v>
+      </c>
+      <c r="V38" t="n">
+        <v>0.3255970400269089</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0.07768306857807052</v>
+      </c>
+      <c r="X38" t="n">
+        <v>0.04093340410763138</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>5104000000</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>7315000000</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>24517000000</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>35244000000</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>109215000000</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>17814000000</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>57453000000</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>32608000000</v>
+      </c>
+      <c r="AG38" t="n">
+        <v>27504000000</v>
+      </c>
+      <c r="AH38" t="n">
+        <v>51110000000</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>1.376277085438419</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>0.6379964781843084</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>3803000000</v>
+      </c>
+      <c r="AL38" t="n">
+        <v>896000000</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>2907000000</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>2200000000</v>
+      </c>
+      <c r="AO38" t="n">
+        <v>1225000000</v>
+      </c>
+      <c r="AP38" t="inlineStr"/>
+      <c r="AQ38" t="n">
+        <v>0.1223639348402576</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>1.105263157894737</v>
+      </c>
+      <c r="AV38" t="n">
+        <v>1745014000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9073,7 +9225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV74"/>
+  <dimension ref="A1:AV75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20068,6 +20220,158 @@
         <v>1747073000</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026 Q2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>quarter</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>12593000000</v>
+      </c>
+      <c r="G75" t="n">
+        <v>5325000000</v>
+      </c>
+      <c r="H75" t="n">
+        <v>7268000000</v>
+      </c>
+      <c r="I75" t="n">
+        <v>892000000</v>
+      </c>
+      <c r="J75" t="n">
+        <v>4025000000</v>
+      </c>
+      <c r="K75" t="n">
+        <v>658000000</v>
+      </c>
+      <c r="L75" t="n">
+        <v>1693000000</v>
+      </c>
+      <c r="M75" t="n">
+        <v>1524000000</v>
+      </c>
+      <c r="N75" t="n">
+        <v>596000000</v>
+      </c>
+      <c r="O75" t="n">
+        <v>928000000</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0.1302279662538144</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>-0.4783586284429455</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0.5771460335106805</v>
+      </c>
+      <c r="S75" t="n">
+        <v>0.1344397681251489</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0.07369173350273962</v>
+      </c>
+      <c r="U75" t="n">
+        <v>0.07083300246168506</v>
+      </c>
+      <c r="V75" t="n">
+        <v>0.3910761154855643</v>
+      </c>
+      <c r="W75" t="n">
+        <v>0.07195820530963158</v>
+      </c>
+      <c r="X75" t="n">
+        <v>0.03380014933255632</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>5104000000</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>7315000000</v>
+      </c>
+      <c r="AA75" t="n">
+        <v>24517000000</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>35244000000</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>109215000000</v>
+      </c>
+      <c r="AD75" t="n">
+        <v>17814000000</v>
+      </c>
+      <c r="AE75" t="n">
+        <v>57453000000</v>
+      </c>
+      <c r="AF75" t="n">
+        <v>32608000000</v>
+      </c>
+      <c r="AG75" t="n">
+        <v>27504000000</v>
+      </c>
+      <c r="AH75" t="n">
+        <v>51110000000</v>
+      </c>
+      <c r="AI75" t="n">
+        <v>1.376277085438419</v>
+      </c>
+      <c r="AJ75" t="n">
+        <v>0.6379964781843084</v>
+      </c>
+      <c r="AK75" t="n">
+        <v>2488000000</v>
+      </c>
+      <c r="AL75" t="n">
+        <v>497000000</v>
+      </c>
+      <c r="AM75" t="n">
+        <v>1991000000</v>
+      </c>
+      <c r="AN75" t="n">
+        <v>1102000000</v>
+      </c>
+      <c r="AO75" t="n">
+        <v>1045000000</v>
+      </c>
+      <c r="AP75" t="inlineStr"/>
+      <c r="AQ75" t="n">
+        <v>0.1581037084094338</v>
+      </c>
+      <c r="AR75" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AS75" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AT75" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AU75" t="n">
+        <v>1.188679245283019</v>
+      </c>
+      <c r="AV75" t="n">
+        <v>1742981000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>